<commit_message>
included pdf export for employee reports and employee records in admin module
</commit_message>
<xml_diff>
--- a/backend/InternTrack_Employees.xlsx
+++ b/backend/InternTrack_Employees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,13 +412,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Bhuvana</v>
+        <v>Admin</v>
       </c>
       <c r="B2" t="str">
-        <v>employee@interntrack.com</v>
+        <v>admin123@gmail.com</v>
       </c>
       <c r="C2" t="str">
-        <v>employee</v>
+        <v>admin</v>
       </c>
     </row>
     <row r="3">
@@ -434,32 +434,32 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Hrithik</v>
+        <v>Mentor</v>
       </c>
       <c r="B4" t="str">
-        <v>hrithik@gmail.com</v>
+        <v>mentor@gmail.com</v>
       </c>
       <c r="C4" t="str">
-        <v>employee</v>
+        <v>mentor</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>admin</v>
+        <v>Mentor2</v>
       </c>
       <c r="B5" t="str">
-        <v>admin123@gmail.com</v>
+        <v>Mentor2@gmail.com</v>
       </c>
       <c r="C5" t="str">
-        <v>admin</v>
+        <v>mentor</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>test</v>
+        <v>Bhuvana</v>
       </c>
       <c r="B6" t="str">
-        <v>test@gmail.com</v>
+        <v>bhuvana@gmail.com</v>
       </c>
       <c r="C6" t="str">
         <v>employee</v>
@@ -467,18 +467,106 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Hrithik</v>
+      </c>
+      <c r="B7" t="str">
+        <v>hrithik@gmail.com</v>
+      </c>
+      <c r="C7" t="str">
+        <v>employee</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Ishani</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ishani@gmail.com</v>
+      </c>
+      <c r="C8" t="str">
+        <v>employee</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Test</v>
+      </c>
+      <c r="B9" t="str">
+        <v>test@gmail.com</v>
+      </c>
+      <c r="C9" t="str">
+        <v>employee</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>hiba</v>
+      </c>
+      <c r="B10" t="str">
+        <v>hiba@gmail.com</v>
+      </c>
+      <c r="C10" t="str">
+        <v>employee</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>sakshi</v>
+      </c>
+      <c r="B11" t="str">
+        <v>sakshi@gmail.com</v>
+      </c>
+      <c r="C11" t="str">
+        <v>employee</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>roshni</v>
+      </c>
+      <c r="B12" t="str">
+        <v>roshni@gmail.com</v>
+      </c>
+      <c r="C12" t="str">
+        <v>employee</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>balaji</v>
+      </c>
+      <c r="B13" t="str">
+        <v>balaji@gmail.com</v>
+      </c>
+      <c r="C13" t="str">
+        <v>employee</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>riyas</v>
+      </c>
+      <c r="B14" t="str">
+        <v>riyas@gmail.com</v>
+      </c>
+      <c r="C14" t="str">
         <v>mentor</v>
       </c>
-      <c r="B7" t="str">
-        <v>mentor@gmail.com</v>
-      </c>
-      <c r="C7" t="str">
-        <v>mentor</v>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>nithin</v>
+      </c>
+      <c r="B15" t="str">
+        <v>nithin@gmail.com</v>
+      </c>
+      <c r="C15" t="str">
+        <v>employee</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
implemented CRUD to PostgreSQL along with month wise and search wise export
</commit_message>
<xml_diff>
--- a/backend/InternTrack_Employees.xlsx
+++ b/backend/InternTrack_Employees.xlsx
@@ -64,8 +64,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,6 +410,18 @@
       <c r="C1" t="str">
         <v>Role</v>
       </c>
+      <c r="D1" t="str">
+        <v>Employment Type</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Department</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Joining Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Status</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -420,6 +433,18 @@
       <c r="C2" t="str">
         <v>admin</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>Administration</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46204.00011574074</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -431,6 +456,18 @@
       <c r="C3" t="str">
         <v>admin</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>Administration</v>
+      </c>
+      <c r="F3" s="1">
+        <v>46204.00011574074</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -442,6 +479,18 @@
       <c r="C4" t="str">
         <v>mentor</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="F4" s="1">
+        <v>46204.00011574074</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -453,6 +502,18 @@
       <c r="C5" t="str">
         <v>mentor</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="F5" s="1">
+        <v>46204.00011574074</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -464,6 +525,18 @@
       <c r="C6" t="str">
         <v>employee</v>
       </c>
+      <c r="D6" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="F6" s="1">
+        <v>46204.00011574074</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -475,6 +548,18 @@
       <c r="C7" t="str">
         <v>employee</v>
       </c>
+      <c r="D7" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="F7" s="1">
+        <v>46204.00011574074</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -486,6 +571,18 @@
       <c r="C8" t="str">
         <v>employee</v>
       </c>
+      <c r="D8" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Operations</v>
+      </c>
+      <c r="F8" s="1">
+        <v>46233.00011574074</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -497,6 +594,18 @@
       <c r="C9" t="str">
         <v>employee</v>
       </c>
+      <c r="D9" t="str">
+        <v>Temporary</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="F9" s="1">
+        <v>46204.00011574074</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Archived</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -508,65 +617,45 @@
       <c r="C10" t="str">
         <v>employee</v>
       </c>
+      <c r="D10" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="F10" s="1">
+        <v>46239.00011574074</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Active</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>sakshi</v>
+        <v>DB TEST</v>
       </c>
       <c r="B11" t="str">
-        <v>sakshi@gmail.com</v>
+        <v>dbtest@email.com</v>
       </c>
       <c r="C11" t="str">
         <v>employee</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>roshni</v>
-      </c>
-      <c r="B12" t="str">
-        <v>roshni@gmail.com</v>
-      </c>
-      <c r="C12" t="str">
-        <v>employee</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>balaji</v>
-      </c>
-      <c r="B13" t="str">
-        <v>balaji@gmail.com</v>
-      </c>
-      <c r="C13" t="str">
-        <v>employee</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>riyas</v>
-      </c>
-      <c r="B14" t="str">
-        <v>riyas@gmail.com</v>
-      </c>
-      <c r="C14" t="str">
-        <v>mentor</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>nithin</v>
-      </c>
-      <c r="B15" t="str">
-        <v>nithin@gmail.com</v>
-      </c>
-      <c r="C15" t="str">
-        <v>employee</v>
+      <c r="D11" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="F11" s="1">
+        <v>46259.00011574074</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>